<commit_message>
Feat: added a kill button for the running process. Fixed the buttons styling as well.
</commit_message>
<xml_diff>
--- a/output.xlsx
+++ b/output.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D16"/>
+  <dimension ref="A1:D3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -441,300 +441,38 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>1300100</t>
+          <t>13401451</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Alice kariuki</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr"/>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>FS_172.23.5.248_HQ_AfEPM_AE_OFFICE, WiFi-Employees, Webmail_2FA_Africa, All, Domain, VPN-Airtel-Employee-G</t>
-        </is>
-      </c>
+          <t>Anthony Ayungo</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>KE-VPN-Employees-Fina</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>1300135</t>
+          <t>13401466</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Freda Mbogori</t>
+          <t>Letoya Mbuthia</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>CicDialer_Reporter, KE-VPN-Employees-CX, KO_AR_DBOs, Ps_Ar, PS_AR_DBOs</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>Cu_Lc_Bi_RW, FS3900_KOINANGE, ke_cu_pl_r, Ke_Cu_PI_R, Cu_Lc_Ne_RW, Dialer_Contacts_IVR_C, Cu_Mc_Ma_Ca_Rw, UniversalWebAccess, Cu_Lc_Ca_Fr_Rw, Ent_Bu_rw, Pl_Ge_RW, Cu_Lc_Sup_R, Cu_Mc_Prj_R, Cu_Lc_Sa_RW, FS_KE_172.23.5.248_AlCu_Lc_Tr_RW, OmniDocsUsers, Cu_Lc_Gen_RW, Cu_Lc_Ce_R, Cu_Mc_Ma_Rw, Cu_Mc_Ma_Op_R, Cu_Lc_In_RW, CSRs, Cu_Mc_Man_Rw, Cu_Lc_Te_RW, Ke_Cu_Oi_R, Cu_Lc_Cr_Ld_Ma_Rw, Cu_Lc_Inf_RW, Air_Ke_BCP_RW, PROXY_KE_OFFICE, Cu_Lc_Pr_RW, KYC_Arc_RW, EPM_KE_OFFICE, Ke_Ns_It_PjTb_R, Cu_Lc_Ce_RW, Vlan_IN, Cu_Lc_Su_RW, Pl_R, Cu_Lc_Fr_Co_Rw, WiFi-Employees, Ke_Fa_Bj_Rw, Webmail_2FA_Africa, Ent_Cor_RW, Ke_Cu_Tim_Tim_RW, Cu_Mc_Ma_Supp_R, Cu_Lc_Cu_Rw, Ke_Ns_Re_R, Cu_Lc_Op_R, Cu_Mc_Re_R, Cu_Lc_Pl_RW, Cu_Lc_RW, Cu_Lc_Re_Rw, M_CustCareArchive, L_Platinum, Cu_Lc_Cr_RW, Cu_Lc_R, Cu_Lc_Ba_Lm_RW, Cu_Lc_Ba_RW, Kencell-Read, Domain, Cu_Mc_Bu_R, Cu_Lc_Int_RW, Cu_Lc_Cc_RW, VPN-Airtel-Employee-GCu_Lc_Ca_RW, CPr_IRC3200N_M, Cu_Lc_Ca_R, Ke_It_CM_RW, Ent_Cre_Co_Cre_RW, Cu_Lc_Fr_RW</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>1300512</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Emeka Oparah</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr"/>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>O365-License-CoPilot EPM_AE_OFFICE, WiFi-Employees, Webmail_2FA_Africa, VIP_EXCO, PROXY_AE_OFFICE_PAC, Domain, VPN-Airtel-Employee-G, PROXY_AE_OFFICE</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>1300553</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Alice Paulsen</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>TZ-VPN-Employees-CX, TZ-VPN-Employees-Mark</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>EPM_TZ_OFFICE, WiFi-Employees, Webmail_2FA_Africa, Domain, PROXY_TZ_OFFICE, VPN-Airtel-Employee-G</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>1300625</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Rose Kamau</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr"/>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>Cu_Lc_Cu_R, ke_cu_pl_r, Ke_Ns_It_PjTb_RW, Ke_Cu_PI_R, Cu_Lc_Sa_R, UniversalWebAccess, Ns_Bu_R, HQ_GT_RW, Cu_Lc_Bi_R, Cu_Lc_In_R, Cu_Mc_Sr_RW, Cu_Lc_Tr_R, Ke_Cu_Scr_RW, Cu_Lc_Int_R, OmniDocsUsers, Cu_M-Csr_Pr_Rw, Cu_Lc_Pr_R, Cu_Lc_Gen_RW, Ke_Ns_Zap_Rw, Cu_Lc_Ce_R, Cu_Mc_Ma_Rw, CSR_CorpWeb_Access_Gr, CSRs, Cu_Lc_Te_RW, Ke_Ma_Rw, Cu_Lc_Cc_R, PROXY_KE_OFFICE, agile_atl_confluence, EPM_AE_OFFICE, Ke_Cu_Sc_RW, Vlan_IN, L_Customer_Care, WiFi-Employees, Webmail_2FA_Africa, Cu_Lc_Sup_RW, Ke_Cu_Tim_Tim_RW, Cu_Lc_Cr_R, Ke_Ns_Re_R, Cu_Lc_Fr_Co_R, Cu_Lc_Op_R, Ke_Cu_Oi_RW, Cu_Lc_Fr_R, Cu_Mc_Pl_RW, Cu_Lc_Ne_R, Cu_Lc_RW, CXO, M_CustCareArchive, Cu_Lc_R, Ke_Zkbp_Rw, Cu_Lc_Pl_R, CCareCitrixUsers, Cu_Mc_Cu_RW, Cu_Mc_Ma_Supp_Rw, CitrixUsers, Cu_Mc_Re_Rw, Customer, Cu_Lc_Ba_RW, Domain, Cu_Mc_Prj_Rw, Cu_Lm_M-Csr_Rw, Cu_Mc_Ma_Ge_Rw, Cu_Lc_Ba_Lm_R, VPN-Airtel-Employee-GKe_Fa_L&amp;D_R, Cu_Lc_Ca_RW, Cu_Lc_Su_R, CPr_IRC3200N_M, Cu_Lc_Ca_R, Cu_Lc_Inf_R, Ke_It_CM_RW, Cu_Lm_Rw, Ke_Comv_Rw</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>1300672</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Mustafa Dhalla</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>KE-VPN-Employees-FinaTZ-VPN-Employees-Fina</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>Finance HQShared, 172.23.7.231-Race-Ra-, FS_TZ_172.27.3.217_GrAllusers, EPM_TZ_OFFICE, WiFi-Employees, Webmail_2FA_Africa, All, 172.23.7.231-Race-BPMFS_TZ_172.27.3.217_Ai, 172.23.7.231-Race-BPMDomain, PROXY_TZ_OFFICE, VPN-Airtel-Employee-G</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>1300954</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>Lydia Kalimunda</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>TZ-VPN-Employees-Sale</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>EPM_TZ_OFFICE, WiFi-Employees, Webmail_2FA_Africa, Domain, PROXY_TZ_OFFICE, VPN-Airtel-Employee-G</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>1301015</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>S�v�rin ONGOUORI</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>GA-VPN-CC, GA-VPN-Employees-IT, GA-VPN-Shop</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>WiFi-Employees, Webmail_2FA_Africa, PROXY_GA_OFFICE, Domain, VPN-Airtel-Employee-GEPM_GA_OFFICE</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>1301223</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>Joujou ILEO NGOYA</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr"/>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>PROXY_CD_OFFICE, Drc-HR-R&amp;W, WiFi-Employees, Webmail_2FA_Africa, VIP_EXCO, Zoom-Host, EPM_CD_OFFICE, Internet_Staff, Domain, ISA_1-6, HR_AF_RW, VPN-Airtel-Employee-G, All, HR_Rw, CD-VPN-Employee-AdminISA_7-18, RWM_RH</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>13012431</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr"/>
-      <c r="C11" t="inlineStr"/>
-      <c r="D11" t="inlineStr"/>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>1301484</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>Lilian Kibiriti</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>TZ-VPN-Employees-Fina</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>FS_TZ_172.27.3.217_MDfinance, EPM_TZ_OFFICE, WiFi-Employees, Webmail_2FA_Africa, Zoom-Host, FS_TZ_172.27.3.217_GrDomain, PROXY_TZ_OFFICE, VPN-Airtel-Employee-G</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>1301682</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>Attawel HAMA</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr"/>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>NE-VPN-EMPLOYEE-SALESEPM_NE_OFFICE, WiFi-Employees, Webmail_2FA_Africa, PROXY_NE_OFFICE, Domain</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>1301742</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>Mwajuma Mbugi</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>TZ-VPN-Employees-Sale</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>EPM_TZ_OFFICE, WiFi-Employees, Webmail_2FA_Africa, FS_TZ_172.27.3.217_s&amp;, Domain, PROXY_TZ_OFFICE, VPN-Airtel-Employee-G</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>1301895</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>Stella Kibacha</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>TZ-VPN-Employees-HR</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>Hr_Ov_Af_Rw, HQ_BCM_SPOCS, Re_Af_RW, HR, finance, EPM_TZ_OFFICE, WiFi-Employees, Webmail_2FA_Africa, VIP_EXCO, Zoom-Host, HQ_To_Co_AI_RW, Domain, PROXY_TZ_OFFICE, VPN-Airtel-Employee-G</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>1302515</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>Sadiq Amako</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
           <t>KE-VPN-Employees-Fina</t>
         </is>
       </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>finance, Allusers, EPM_AE_OFFICE, WiFi-Employees, Webmail_2FA_Africa, PROXY_AE_OFFICE_PAC, Domain, VPN-Airtel-Employee-G, PROXY_AE_OFFICE, FS_KE_172.23.5.248_Ta</t>
-        </is>
-      </c>
+      <c r="D3" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>